<commit_message>
minor fix on error messages
</commit_message>
<xml_diff>
--- a/models/test_data_IZ_to_IZ.xlsx
+++ b/models/test_data_IZ_to_IZ.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\projects\iz_to_iz_transfer\models\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC8B217A-9589-4647-8416-B015B47E4C28}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7611C47-C781-491E-AAF6-D81940B5D130}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2295" yWindow="2295" windowWidth="21600" windowHeight="12645" tabRatio="800" xr2:uid="{AD365A3D-3304-46D8-98A5-452209B6D1C5}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" tabRatio="800" xr2:uid="{AD365A3D-3304-46D8-98A5-452209B6D1C5}"/>
   </bookViews>
   <sheets>
     <sheet name="General" sheetId="1" r:id="rId1"/>
@@ -1105,7 +1105,7 @@
         <v>143</v>
       </c>
       <c r="B20" s="3">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="C20" t="s">
         <v>144</v>

</xml_diff>

<commit_message>
add update processes for items
</commit_message>
<xml_diff>
--- a/models/test_data_IZ_to_IZ.xlsx
+++ b/models/test_data_IZ_to_IZ.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\projects\iz_to_iz_transfer\models\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA5E594A-B813-4F06-A155-D5A2F43723B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6568222-5C60-4480-81E5-2BC8EB4E24C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" tabRatio="800" activeTab="2" xr2:uid="{AD365A3D-3304-46D8-98A5-452209B6D1C5}"/>
+    <workbookView xWindow="3120" yWindow="3120" windowWidth="21600" windowHeight="12645" tabRatio="800" xr2:uid="{AD365A3D-3304-46D8-98A5-452209B6D1C5}"/>
   </bookViews>
   <sheets>
     <sheet name="General" sheetId="1" r:id="rId1"/>
@@ -1108,7 +1108,7 @@
         <v>143</v>
       </c>
       <c r="B20" s="3">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C20" t="s">
         <v>144</v>

</xml_diff>